<commit_message>
debug vgrf prediction mapping issue
</commit_message>
<xml_diff>
--- a/results/ncbc_s10/TM_p6/pred_peaks.xlsx
+++ b/results/ncbc_s10/TM_p6/pred_peaks.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C325"/>
+  <dimension ref="A1:C296"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -455,7 +455,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1.017782688140869</v>
+        <v>1.019579887390137</v>
       </c>
     </row>
     <row r="3">
@@ -468,7 +468,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1.011259794235229</v>
+        <v>1.107705354690552</v>
       </c>
     </row>
     <row r="4">
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1.085390090942383</v>
+        <v>1.085720896720886</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1.244743824005127</v>
+        <v>1.191529273986816</v>
       </c>
     </row>
     <row r="6">
@@ -507,7 +507,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1.453410983085632</v>
+        <v>1.404990911483765</v>
       </c>
     </row>
     <row r="7">
@@ -520,7 +520,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1.587252855300903</v>
+        <v>1.381601929664612</v>
       </c>
     </row>
     <row r="8">
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1.572365283966064</v>
+        <v>1.457111001014709</v>
       </c>
     </row>
     <row r="9">
@@ -546,7 +546,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1.489366769790649</v>
+        <v>1.447875022888184</v>
       </c>
     </row>
     <row r="10">
@@ -559,7 +559,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1.583930015563965</v>
+        <v>1.407451033592224</v>
       </c>
     </row>
     <row r="11">
@@ -572,7 +572,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1.473952054977417</v>
+        <v>1.493628859519958</v>
       </c>
     </row>
     <row r="12">
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1.663620233535767</v>
+        <v>1.515350818634033</v>
       </c>
     </row>
     <row r="13">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1.614044070243835</v>
+        <v>1.456912159919739</v>
       </c>
     </row>
     <row r="14">
@@ -611,7 +611,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1.538431406021118</v>
+        <v>1.475498557090759</v>
       </c>
     </row>
     <row r="15">
@@ -624,7 +624,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1.634886145591736</v>
+        <v>1.462712168693542</v>
       </c>
     </row>
     <row r="16">
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1.583720803260803</v>
+        <v>1.456510305404663</v>
       </c>
     </row>
     <row r="17">
@@ -650,7 +650,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1.610547423362732</v>
+        <v>1.480282783508301</v>
       </c>
     </row>
     <row r="18">
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1.617512941360474</v>
+        <v>1.471338272094727</v>
       </c>
     </row>
     <row r="19">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1.627564668655396</v>
+        <v>1.420951366424561</v>
       </c>
     </row>
     <row r="20">
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1.645364165306091</v>
+        <v>1.49280047416687</v>
       </c>
     </row>
     <row r="21">
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1.62424623966217</v>
+        <v>1.472285509109497</v>
       </c>
     </row>
     <row r="22">
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1.657349944114685</v>
+        <v>1.49890923500061</v>
       </c>
     </row>
     <row r="23">
@@ -728,7 +728,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1.64026939868927</v>
+        <v>1.501019716262817</v>
       </c>
     </row>
     <row r="24">
@@ -741,7 +741,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1.680082678794861</v>
+        <v>1.517808437347412</v>
       </c>
     </row>
     <row r="25">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1.646951913833618</v>
+        <v>1.461048364639282</v>
       </c>
     </row>
     <row r="26">
@@ -767,7 +767,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1.675243496894836</v>
+        <v>1.523648262023926</v>
       </c>
     </row>
     <row r="27">
@@ -780,7 +780,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1.596617341041565</v>
+        <v>1.440815210342407</v>
       </c>
     </row>
     <row r="28">
@@ -793,7 +793,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1.646086692810059</v>
+        <v>1.48432993888855</v>
       </c>
     </row>
     <row r="29">
@@ -806,7 +806,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1.691328883171082</v>
+        <v>1.423485159873962</v>
       </c>
     </row>
     <row r="30">
@@ -819,7 +819,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1.525837898254395</v>
+        <v>1.451815843582153</v>
       </c>
     </row>
     <row r="31">
@@ -832,7 +832,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1.487819910049438</v>
+        <v>1.427202701568604</v>
       </c>
     </row>
     <row r="32">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1.591235756874084</v>
+        <v>1.473775386810303</v>
       </c>
     </row>
     <row r="33">
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1.684960126876831</v>
+        <v>1.488567352294922</v>
       </c>
     </row>
     <row r="34">
@@ -871,7 +871,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1.621328353881836</v>
+        <v>1.465397715568542</v>
       </c>
     </row>
     <row r="35">
@@ -884,7 +884,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1.66678261756897</v>
+        <v>1.46942925453186</v>
       </c>
     </row>
     <row r="36">
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1.669066548347473</v>
+        <v>1.335006237030029</v>
       </c>
     </row>
     <row r="37">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1.673089981079102</v>
+        <v>1.431967496871948</v>
       </c>
     </row>
     <row r="38">
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1.639109134674072</v>
+        <v>1.415957450866699</v>
       </c>
     </row>
     <row r="39">
@@ -936,7 +936,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1.66305685043335</v>
+        <v>1.429287672042847</v>
       </c>
     </row>
     <row r="40">
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>1.637229323387146</v>
+        <v>1.371182918548584</v>
       </c>
     </row>
     <row r="41">
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1.639355182647705</v>
+        <v>1.388138294219971</v>
       </c>
     </row>
     <row r="42">
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1.672861814498901</v>
+        <v>1.49602198600769</v>
       </c>
     </row>
     <row r="43">
@@ -988,7 +988,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1.650144219398499</v>
+        <v>1.398633122444153</v>
       </c>
     </row>
     <row r="44">
@@ -1001,7 +1001,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>1.491280794143677</v>
+        <v>1.503104209899902</v>
       </c>
     </row>
     <row r="45">
@@ -1014,7 +1014,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1.6762615442276</v>
+        <v>1.412479162216187</v>
       </c>
     </row>
     <row r="46">
@@ -1027,7 +1027,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1.700748682022095</v>
+        <v>1.437423706054688</v>
       </c>
     </row>
     <row r="47">
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1.669358611106873</v>
+        <v>1.441995859146118</v>
       </c>
     </row>
     <row r="48">
@@ -1053,7 +1053,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>1.657749772071838</v>
+        <v>1.44147253036499</v>
       </c>
     </row>
     <row r="49">
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1.648998618125916</v>
+        <v>1.47114109992981</v>
       </c>
     </row>
     <row r="50">
@@ -1079,7 +1079,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>1.52126133441925</v>
+        <v>1.473813891410828</v>
       </c>
     </row>
     <row r="51">
@@ -1092,7 +1092,7 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>1.643142700195312</v>
+        <v>1.448682904243469</v>
       </c>
     </row>
     <row r="52">
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>1.669290542602539</v>
+        <v>1.404899120330811</v>
       </c>
     </row>
     <row r="53">
@@ -1118,7 +1118,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1.610885620117188</v>
+        <v>1.423952221870422</v>
       </c>
     </row>
     <row r="54">
@@ -1131,7 +1131,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1.620854496955872</v>
+        <v>1.439913868904114</v>
       </c>
     </row>
     <row r="55">
@@ -1144,7 +1144,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1.520437717437744</v>
+        <v>1.465478420257568</v>
       </c>
     </row>
     <row r="56">
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>1.608694314956665</v>
+        <v>1.474416971206665</v>
       </c>
     </row>
     <row r="57">
@@ -1170,7 +1170,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>1.572484493255615</v>
+        <v>1.427802085876465</v>
       </c>
     </row>
     <row r="58">
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>1.679720878601074</v>
+        <v>1.408345460891724</v>
       </c>
     </row>
     <row r="59">
@@ -1196,7 +1196,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>1.630383610725403</v>
+        <v>1.453164339065552</v>
       </c>
     </row>
     <row r="60">
@@ -1209,7 +1209,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1.586873650550842</v>
+        <v>1.476725578308105</v>
       </c>
     </row>
     <row r="61">
@@ -1222,7 +1222,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1.530810832977295</v>
+        <v>1.354921579360962</v>
       </c>
     </row>
     <row r="62">
@@ -1235,7 +1235,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1.590811610221863</v>
+        <v>1.408491849899292</v>
       </c>
     </row>
     <row r="63">
@@ -1248,7 +1248,7 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>1.577479362487793</v>
+        <v>1.457629203796387</v>
       </c>
     </row>
     <row r="64">
@@ -1261,7 +1261,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1.432181596755981</v>
+        <v>1.351901650428772</v>
       </c>
     </row>
     <row r="65">
@@ -1274,7 +1274,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>1.468499183654785</v>
+        <v>1.440387725830078</v>
       </c>
     </row>
     <row r="66">
@@ -1287,7 +1287,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1.547367453575134</v>
+        <v>1.47491717338562</v>
       </c>
     </row>
     <row r="67">
@@ -1300,7 +1300,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>1.558165550231934</v>
+        <v>1.343902707099915</v>
       </c>
     </row>
     <row r="68">
@@ -1313,7 +1313,7 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>1.448744893074036</v>
+        <v>1.394290924072266</v>
       </c>
     </row>
     <row r="69">
@@ -1326,7 +1326,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>1.498350143432617</v>
+        <v>1.428834438323975</v>
       </c>
     </row>
     <row r="70">
@@ -1339,7 +1339,7 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>1.602278590202332</v>
+        <v>1.43763256072998</v>
       </c>
     </row>
     <row r="71">
@@ -1352,7 +1352,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>1.54930591583252</v>
+        <v>1.508557319641113</v>
       </c>
     </row>
     <row r="72">
@@ -1365,7 +1365,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1.632749438285828</v>
+        <v>1.399560213088989</v>
       </c>
     </row>
     <row r="73">
@@ -1378,7 +1378,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>1.626356720924377</v>
+        <v>1.451844096183777</v>
       </c>
     </row>
     <row r="74">
@@ -1391,7 +1391,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>1.616389751434326</v>
+        <v>1.34053373336792</v>
       </c>
     </row>
     <row r="75">
@@ -1404,7 +1404,7 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>1.634220957756042</v>
+        <v>1.45723021030426</v>
       </c>
     </row>
     <row r="76">
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>1.628300547599792</v>
+        <v>1.594358682632446</v>
       </c>
     </row>
     <row r="77">
@@ -1430,7 +1430,7 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>1.501736879348755</v>
+        <v>1.410530567169189</v>
       </c>
     </row>
     <row r="78">
@@ -1443,7 +1443,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>1.515017509460449</v>
+        <v>1.441631317138672</v>
       </c>
     </row>
     <row r="79">
@@ -1456,7 +1456,7 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>1.599318981170654</v>
+        <v>1.399919033050537</v>
       </c>
     </row>
     <row r="80">
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>1.648612141609192</v>
+        <v>1.481651782989502</v>
       </c>
     </row>
     <row r="81">
@@ -1482,7 +1482,7 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>1.546343564987183</v>
+        <v>1.46237325668335</v>
       </c>
     </row>
     <row r="82">
@@ -1495,7 +1495,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>1.561737060546875</v>
+        <v>1.441887855529785</v>
       </c>
     </row>
     <row r="83">
@@ -1508,7 +1508,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>1.573513150215149</v>
+        <v>1.425744771957397</v>
       </c>
     </row>
     <row r="84">
@@ -1521,7 +1521,7 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>1.443772792816162</v>
+        <v>1.439502239227295</v>
       </c>
     </row>
     <row r="85">
@@ -1534,7 +1534,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>1.641269087791443</v>
+        <v>1.531932830810547</v>
       </c>
     </row>
     <row r="86">
@@ -1547,7 +1547,7 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>1.643048763275146</v>
+        <v>1.472862958908081</v>
       </c>
     </row>
     <row r="87">
@@ -1560,7 +1560,7 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>1.599284648895264</v>
+        <v>1.452461004257202</v>
       </c>
     </row>
     <row r="88">
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>1.640777111053467</v>
+        <v>1.470597743988037</v>
       </c>
     </row>
     <row r="89">
@@ -1586,7 +1586,7 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>1.460995674133301</v>
+        <v>1.462612748146057</v>
       </c>
     </row>
     <row r="90">
@@ -1599,7 +1599,7 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>1.610651254653931</v>
+        <v>1.394681692123413</v>
       </c>
     </row>
     <row r="91">
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>1.553707838058472</v>
+        <v>1.430570125579834</v>
       </c>
     </row>
     <row r="92">
@@ -1625,7 +1625,7 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>1.551201105117798</v>
+        <v>1.508414626121521</v>
       </c>
     </row>
     <row r="93">
@@ -1638,7 +1638,7 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>1.552949905395508</v>
+        <v>1.492284297943115</v>
       </c>
     </row>
     <row r="94">
@@ -1651,7 +1651,7 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>1.501465797424316</v>
+        <v>1.449597716331482</v>
       </c>
     </row>
     <row r="95">
@@ -1664,7 +1664,7 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>1.640299677848816</v>
+        <v>1.454996109008789</v>
       </c>
     </row>
     <row r="96">
@@ -1677,7 +1677,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>1.377951383590698</v>
+        <v>1.407389521598816</v>
       </c>
     </row>
     <row r="97">
@@ -1690,7 +1690,7 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>1.461437463760376</v>
+        <v>1.344988346099854</v>
       </c>
     </row>
     <row r="98">
@@ -1703,7 +1703,7 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>1.440449476242065</v>
+        <v>1.442939877510071</v>
       </c>
     </row>
     <row r="99">
@@ -1716,7 +1716,7 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>1.566853284835815</v>
+        <v>1.497887849807739</v>
       </c>
     </row>
     <row r="100">
@@ -1729,7 +1729,7 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>1.505176544189453</v>
+        <v>1.455919027328491</v>
       </c>
     </row>
     <row r="101">
@@ -1742,7 +1742,7 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>1.617632865905762</v>
+        <v>1.492055416107178</v>
       </c>
     </row>
     <row r="102">
@@ -1755,7 +1755,7 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>1.636105179786682</v>
+        <v>1.387318134307861</v>
       </c>
     </row>
     <row r="103">
@@ -1768,7 +1768,7 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>1.634537100791931</v>
+        <v>1.482232928276062</v>
       </c>
     </row>
     <row r="104">
@@ -1781,7 +1781,7 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>1.623638272285461</v>
+        <v>1.415198683738708</v>
       </c>
     </row>
     <row r="105">
@@ -1794,7 +1794,7 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>1.594157457351685</v>
+        <v>1.485689640045166</v>
       </c>
     </row>
     <row r="106">
@@ -1807,7 +1807,7 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>1.577037453651428</v>
+        <v>1.397347927093506</v>
       </c>
     </row>
     <row r="107">
@@ -1820,7 +1820,7 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>1.659572124481201</v>
+        <v>1.438451647758484</v>
       </c>
     </row>
     <row r="108">
@@ -1833,7 +1833,7 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>1.501839160919189</v>
+        <v>1.399697542190552</v>
       </c>
     </row>
     <row r="109">
@@ -1846,7 +1846,7 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>1.640473484992981</v>
+        <v>1.453266859054565</v>
       </c>
     </row>
     <row r="110">
@@ -1859,7 +1859,7 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>1.571383357048035</v>
+        <v>1.456573247909546</v>
       </c>
     </row>
     <row r="111">
@@ -1872,7 +1872,7 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>1.567179441452026</v>
+        <v>1.42725682258606</v>
       </c>
     </row>
     <row r="112">
@@ -1885,7 +1885,7 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>1.512376666069031</v>
+        <v>1.429110288619995</v>
       </c>
     </row>
     <row r="113">
@@ -1898,7 +1898,7 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>1.580183267593384</v>
+        <v>1.420335054397583</v>
       </c>
     </row>
     <row r="114">
@@ -1911,7 +1911,7 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>1.591456532478333</v>
+        <v>1.458113074302673</v>
       </c>
     </row>
     <row r="115">
@@ -1924,7 +1924,7 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>1.634092092514038</v>
+        <v>1.416089534759521</v>
       </c>
     </row>
     <row r="116">
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>1.581115961074829</v>
+        <v>1.468939065933228</v>
       </c>
     </row>
     <row r="117">
@@ -1950,7 +1950,7 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>1.579591512680054</v>
+        <v>1.366449356079102</v>
       </c>
     </row>
     <row r="118">
@@ -1963,7 +1963,7 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>1.60157299041748</v>
+        <v>1.347291111946106</v>
       </c>
     </row>
     <row r="119">
@@ -1976,7 +1976,7 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>1.635728240013123</v>
+        <v>1.405141949653625</v>
       </c>
     </row>
     <row r="120">
@@ -1989,7 +1989,7 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>1.570778012275696</v>
+        <v>1.450339674949646</v>
       </c>
     </row>
     <row r="121">
@@ -2002,7 +2002,7 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>1.488328695297241</v>
+        <v>1.439679861068726</v>
       </c>
     </row>
     <row r="122">
@@ -2015,7 +2015,7 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>1.535593032836914</v>
+        <v>1.439709067344666</v>
       </c>
     </row>
     <row r="123">
@@ -2028,7 +2028,7 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>1.539654731750488</v>
+        <v>1.450636625289917</v>
       </c>
     </row>
     <row r="124">
@@ -2041,7 +2041,7 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>1.578756332397461</v>
+        <v>1.427162408828735</v>
       </c>
     </row>
     <row r="125">
@@ -2054,7 +2054,7 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>1.633102536201477</v>
+        <v>1.456133246421814</v>
       </c>
     </row>
     <row r="126">
@@ -2067,7 +2067,7 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>1.533387184143066</v>
+        <v>1.439695715904236</v>
       </c>
     </row>
     <row r="127">
@@ -2080,7 +2080,7 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>1.622321844100952</v>
+        <v>1.478324770927429</v>
       </c>
     </row>
     <row r="128">
@@ -2093,7 +2093,7 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>1.445369958877563</v>
+        <v>1.422887802124023</v>
       </c>
     </row>
     <row r="129">
@@ -2106,7 +2106,7 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>1.514252662658691</v>
+        <v>1.446035623550415</v>
       </c>
     </row>
     <row r="130">
@@ -2119,7 +2119,7 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>1.576484441757202</v>
+        <v>1.397491335868835</v>
       </c>
     </row>
     <row r="131">
@@ -2132,7 +2132,7 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>1.486977577209473</v>
+        <v>1.389269828796387</v>
       </c>
     </row>
     <row r="132">
@@ -2145,7 +2145,7 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>1.516575455665588</v>
+        <v>1.468173265457153</v>
       </c>
     </row>
     <row r="133">
@@ -2158,7 +2158,7 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>1.538959860801697</v>
+        <v>1.422892451286316</v>
       </c>
     </row>
     <row r="134">
@@ -2171,7 +2171,7 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>1.551610469818115</v>
+        <v>1.437733173370361</v>
       </c>
     </row>
     <row r="135">
@@ -2184,7 +2184,7 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>1.496017217636108</v>
+        <v>1.433385252952576</v>
       </c>
     </row>
     <row r="136">
@@ -2197,7 +2197,7 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>1.633423805236816</v>
+        <v>1.408397197723389</v>
       </c>
     </row>
     <row r="137">
@@ -2210,7 +2210,7 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>1.594168186187744</v>
+        <v>1.30051052570343</v>
       </c>
     </row>
     <row r="138">
@@ -2223,7 +2223,7 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>1.464774012565613</v>
+        <v>1.477584838867188</v>
       </c>
     </row>
     <row r="139">
@@ -2236,7 +2236,7 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>1.584601283073425</v>
+        <v>1.505982756614685</v>
       </c>
     </row>
     <row r="140">
@@ -2249,7 +2249,7 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>1.571929693222046</v>
+        <v>1.418157339096069</v>
       </c>
     </row>
     <row r="141">
@@ -2262,7 +2262,7 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>1.603219985961914</v>
+        <v>1.42559027671814</v>
       </c>
     </row>
     <row r="142">
@@ -2275,7 +2275,7 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>1.464363813400269</v>
+        <v>1.353667259216309</v>
       </c>
     </row>
     <row r="143">
@@ -2288,7 +2288,7 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>1.622429370880127</v>
+        <v>1.424566149711609</v>
       </c>
     </row>
     <row r="144">
@@ -2301,7 +2301,7 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>1.543646216392517</v>
+        <v>1.385576725006104</v>
       </c>
     </row>
     <row r="145">
@@ -2314,7 +2314,7 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>1.600255727767944</v>
+        <v>1.225486755371094</v>
       </c>
     </row>
     <row r="146">
@@ -2327,7 +2327,7 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>1.532732605934143</v>
+        <v>1.096878528594971</v>
       </c>
     </row>
     <row r="147">
@@ -2340,7 +2340,7 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>1.474379420280457</v>
+        <v>1.127435922622681</v>
       </c>
     </row>
     <row r="148">
@@ -2353,194 +2353,194 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>1.534609317779541</v>
+        <v>0.9994391202926636</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
-        <v>147</v>
+        <v>0</v>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>1.514198780059814</v>
+        <v>0.9888131618499756</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
-        <v>148</v>
+        <v>1</v>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>1.604749441146851</v>
+        <v>0.9755783677101135</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>149</v>
+        <v>2</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>1.607508897781372</v>
+        <v>1.061368346214294</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
-        <v>150</v>
+        <v>3</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>1.502472758293152</v>
+        <v>1.223720550537109</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>151</v>
+        <v>4</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>1.463840007781982</v>
+        <v>1.48204493522644</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>152</v>
+        <v>5</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>1.513511180877686</v>
+        <v>1.514732956886292</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
-        <v>153</v>
+        <v>6</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>1.597021579742432</v>
+        <v>1.430176258087158</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>154</v>
+        <v>7</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>1.621070265769958</v>
+        <v>1.424416065216064</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>155</v>
+        <v>8</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>1.622893810272217</v>
+        <v>1.440253853797913</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>156</v>
+        <v>9</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>1.451763868331909</v>
+        <v>1.446954011917114</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
-        <v>157</v>
+        <v>10</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>1.341675996780396</v>
+        <v>1.422994017601013</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
-        <v>158</v>
+        <v>11</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>1.130985498428345</v>
+        <v>1.41388463973999</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
-        <v>159</v>
+        <v>12</v>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>1.367464184761047</v>
+        <v>1.484577059745789</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
-        <v>160</v>
+        <v>13</v>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>0.9923443198204041</v>
+        <v>1.410073161125183</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="B163" t="inlineStr">
         <is>
@@ -2548,12 +2548,12 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>0.9914367198944092</v>
+        <v>1.431210279464722</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="B164" t="inlineStr">
         <is>
@@ -2561,12 +2561,12 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>1.056403636932373</v>
+        <v>1.422250747680664</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="B165" t="inlineStr">
         <is>
@@ -2574,12 +2574,12 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>1.117297053337097</v>
+        <v>1.364811182022095</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="B166" t="inlineStr">
         <is>
@@ -2587,12 +2587,12 @@
         </is>
       </c>
       <c r="C166" t="n">
-        <v>1.084017276763916</v>
+        <v>1.477779269218445</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="B167" t="inlineStr">
         <is>
@@ -2600,12 +2600,12 @@
         </is>
       </c>
       <c r="C167" t="n">
-        <v>1.167728185653687</v>
+        <v>1.426172971725464</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="B168" t="inlineStr">
         <is>
@@ -2613,12 +2613,12 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>1.487370491027832</v>
+        <v>1.414201736450195</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="B169" t="inlineStr">
         <is>
@@ -2626,12 +2626,12 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>1.52350115776062</v>
+        <v>1.392321586608887</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="B170" t="inlineStr">
         <is>
@@ -2639,12 +2639,12 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>1.570776581764221</v>
+        <v>1.433545351028442</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="B171" t="inlineStr">
         <is>
@@ -2652,12 +2652,12 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>1.544726490974426</v>
+        <v>1.499427080154419</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="B172" t="inlineStr">
         <is>
@@ -2665,12 +2665,12 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>1.42765748500824</v>
+        <v>1.399299144744873</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="B173" t="inlineStr">
         <is>
@@ -2678,12 +2678,12 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>1.523399114608765</v>
+        <v>1.461203813552856</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="B174" t="inlineStr">
         <is>
@@ -2691,12 +2691,12 @@
         </is>
       </c>
       <c r="C174" t="n">
-        <v>1.474546790122986</v>
+        <v>1.390862703323364</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="B175" t="inlineStr">
         <is>
@@ -2704,12 +2704,12 @@
         </is>
       </c>
       <c r="C175" t="n">
-        <v>1.378845930099487</v>
+        <v>1.375313282012939</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="B176" t="inlineStr">
         <is>
@@ -2717,12 +2717,12 @@
         </is>
       </c>
       <c r="C176" t="n">
-        <v>1.474708676338196</v>
+        <v>1.432182550430298</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="B177" t="inlineStr">
         <is>
@@ -2730,12 +2730,12 @@
         </is>
       </c>
       <c r="C177" t="n">
-        <v>1.554271101951599</v>
+        <v>1.457907199859619</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="B178" t="inlineStr">
         <is>
@@ -2743,12 +2743,12 @@
         </is>
       </c>
       <c r="C178" t="n">
-        <v>1.624341607093811</v>
+        <v>1.38600492477417</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
@@ -2756,12 +2756,12 @@
         </is>
       </c>
       <c r="C179" t="n">
-        <v>1.576879739761353</v>
+        <v>1.413287758827209</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="B180" t="inlineStr">
         <is>
@@ -2769,12 +2769,12 @@
         </is>
       </c>
       <c r="C180" t="n">
-        <v>1.499188899993896</v>
+        <v>1.395279884338379</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
@@ -2782,12 +2782,12 @@
         </is>
       </c>
       <c r="C181" t="n">
-        <v>1.476046323776245</v>
+        <v>1.38740074634552</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
@@ -2795,12 +2795,12 @@
         </is>
       </c>
       <c r="C182" t="n">
-        <v>1.451681613922119</v>
+        <v>1.405502557754517</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="B183" t="inlineStr">
         <is>
@@ -2808,12 +2808,12 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>1.48565149307251</v>
+        <v>1.500025987625122</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="B184" t="inlineStr">
         <is>
@@ -2821,12 +2821,12 @@
         </is>
       </c>
       <c r="C184" t="n">
-        <v>1.40953254699707</v>
+        <v>1.415626525878906</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="B185" t="inlineStr">
         <is>
@@ -2834,12 +2834,12 @@
         </is>
       </c>
       <c r="C185" t="n">
-        <v>1.534208536148071</v>
+        <v>1.509721279144287</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
@@ -2847,12 +2847,12 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>1.447814464569092</v>
+        <v>1.481805086135864</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
@@ -2860,12 +2860,12 @@
         </is>
       </c>
       <c r="C187" t="n">
-        <v>1.588563561439514</v>
+        <v>1.52589213848114</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="B188" t="inlineStr">
         <is>
@@ -2873,12 +2873,12 @@
         </is>
       </c>
       <c r="C188" t="n">
-        <v>1.613664388656616</v>
+        <v>1.566524505615234</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
@@ -2886,12 +2886,12 @@
         </is>
       </c>
       <c r="C189" t="n">
-        <v>1.496647000312805</v>
+        <v>1.431832790374756</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
@@ -2899,12 +2899,12 @@
         </is>
       </c>
       <c r="C190" t="n">
-        <v>1.537810444831848</v>
+        <v>1.53935182094574</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="B191" t="inlineStr">
         <is>
@@ -2912,12 +2912,12 @@
         </is>
       </c>
       <c r="C191" t="n">
-        <v>1.471099019050598</v>
+        <v>1.455713748931885</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
@@ -2925,12 +2925,12 @@
         </is>
       </c>
       <c r="C192" t="n">
-        <v>1.696041464805603</v>
+        <v>1.476786971092224</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="B193" t="inlineStr">
         <is>
@@ -2938,12 +2938,12 @@
         </is>
       </c>
       <c r="C193" t="n">
-        <v>1.645030975341797</v>
+        <v>1.404298305511475</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
@@ -2951,12 +2951,12 @@
         </is>
       </c>
       <c r="C194" t="n">
-        <v>1.418500185012817</v>
+        <v>1.445971965789795</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="B195" t="inlineStr">
         <is>
@@ -2964,12 +2964,12 @@
         </is>
       </c>
       <c r="C195" t="n">
-        <v>1.555674076080322</v>
+        <v>1.435760855674744</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="B196" t="inlineStr">
         <is>
@@ -2977,12 +2977,12 @@
         </is>
       </c>
       <c r="C196" t="n">
-        <v>1.557124614715576</v>
+        <v>1.472887277603149</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="n">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="B197" t="inlineStr">
         <is>
@@ -2990,12 +2990,12 @@
         </is>
       </c>
       <c r="C197" t="n">
-        <v>1.502175807952881</v>
+        <v>1.335937023162842</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="n">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="B198" t="inlineStr">
         <is>
@@ -3003,12 +3003,12 @@
         </is>
       </c>
       <c r="C198" t="n">
-        <v>1.516951322555542</v>
+        <v>1.410462498664856</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="n">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="B199" t="inlineStr">
         <is>
@@ -3016,12 +3016,12 @@
         </is>
       </c>
       <c r="C199" t="n">
-        <v>1.480602502822876</v>
+        <v>1.412007570266724</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="n">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="B200" t="inlineStr">
         <is>
@@ -3029,12 +3029,12 @@
         </is>
       </c>
       <c r="C200" t="n">
-        <v>1.61355459690094</v>
+        <v>1.501421689987183</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="n">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="B201" t="inlineStr">
         <is>
@@ -3042,12 +3042,12 @@
         </is>
       </c>
       <c r="C201" t="n">
-        <v>1.484200358390808</v>
+        <v>1.412474513053894</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="n">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="B202" t="inlineStr">
         <is>
@@ -3055,12 +3055,12 @@
         </is>
       </c>
       <c r="C202" t="n">
-        <v>1.483416795730591</v>
+        <v>1.470696449279785</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="n">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="B203" t="inlineStr">
         <is>
@@ -3068,12 +3068,12 @@
         </is>
       </c>
       <c r="C203" t="n">
-        <v>1.612298846244812</v>
+        <v>1.368030309677124</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="n">
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="B204" t="inlineStr">
         <is>
@@ -3081,12 +3081,12 @@
         </is>
       </c>
       <c r="C204" t="n">
-        <v>1.499248147010803</v>
+        <v>1.385962605476379</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="n">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="B205" t="inlineStr">
         <is>
@@ -3094,12 +3094,12 @@
         </is>
       </c>
       <c r="C205" t="n">
-        <v>1.539684534072876</v>
+        <v>1.34205961227417</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="n">
-        <v>43</v>
+        <v>57</v>
       </c>
       <c r="B206" t="inlineStr">
         <is>
@@ -3107,12 +3107,12 @@
         </is>
       </c>
       <c r="C206" t="n">
-        <v>1.580992460250854</v>
+        <v>1.3685142993927</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="n">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="B207" t="inlineStr">
         <is>
@@ -3120,12 +3120,12 @@
         </is>
       </c>
       <c r="C207" t="n">
-        <v>1.464502811431885</v>
+        <v>1.449473738670349</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="B208" t="inlineStr">
         <is>
@@ -3133,12 +3133,12 @@
         </is>
       </c>
       <c r="C208" t="n">
-        <v>1.63696825504303</v>
+        <v>1.3921058177948</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="n">
-        <v>46</v>
+        <v>60</v>
       </c>
       <c r="B209" t="inlineStr">
         <is>
@@ -3146,12 +3146,12 @@
         </is>
       </c>
       <c r="C209" t="n">
-        <v>1.529585123062134</v>
+        <v>1.395275473594666</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="n">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="B210" t="inlineStr">
         <is>
@@ -3159,12 +3159,12 @@
         </is>
       </c>
       <c r="C210" t="n">
-        <v>1.623012781143188</v>
+        <v>1.394354104995728</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="n">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="B211" t="inlineStr">
         <is>
@@ -3172,12 +3172,12 @@
         </is>
       </c>
       <c r="C211" t="n">
-        <v>1.557936429977417</v>
+        <v>1.404058456420898</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="n">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="B212" t="inlineStr">
         <is>
@@ -3185,12 +3185,12 @@
         </is>
       </c>
       <c r="C212" t="n">
-        <v>1.646969079971313</v>
+        <v>1.495849609375</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="n">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="B213" t="inlineStr">
         <is>
@@ -3198,12 +3198,12 @@
         </is>
       </c>
       <c r="C213" t="n">
-        <v>1.371405005455017</v>
+        <v>1.463335156440735</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="n">
-        <v>51</v>
+        <v>65</v>
       </c>
       <c r="B214" t="inlineStr">
         <is>
@@ -3211,12 +3211,12 @@
         </is>
       </c>
       <c r="C214" t="n">
-        <v>1.560373544692993</v>
+        <v>1.428042054176331</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="n">
-        <v>52</v>
+        <v>66</v>
       </c>
       <c r="B215" t="inlineStr">
         <is>
@@ -3224,12 +3224,12 @@
         </is>
       </c>
       <c r="C215" t="n">
-        <v>1.454337000846863</v>
+        <v>1.40077805519104</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="n">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="B216" t="inlineStr">
         <is>
@@ -3237,12 +3237,12 @@
         </is>
       </c>
       <c r="C216" t="n">
-        <v>1.603435158729553</v>
+        <v>1.374676465988159</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="n">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="B217" t="inlineStr">
         <is>
@@ -3250,12 +3250,12 @@
         </is>
       </c>
       <c r="C217" t="n">
-        <v>1.576144218444824</v>
+        <v>1.417614221572876</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="n">
-        <v>55</v>
+        <v>69</v>
       </c>
       <c r="B218" t="inlineStr">
         <is>
@@ -3263,12 +3263,12 @@
         </is>
       </c>
       <c r="C218" t="n">
-        <v>1.587984561920166</v>
+        <v>1.458158254623413</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="n">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="B219" t="inlineStr">
         <is>
@@ -3276,12 +3276,12 @@
         </is>
       </c>
       <c r="C219" t="n">
-        <v>1.549557447433472</v>
+        <v>1.484405994415283</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="n">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="B220" t="inlineStr">
         <is>
@@ -3289,12 +3289,12 @@
         </is>
       </c>
       <c r="C220" t="n">
-        <v>1.699130177497864</v>
+        <v>1.378488063812256</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="B221" t="inlineStr">
         <is>
@@ -3302,12 +3302,12 @@
         </is>
       </c>
       <c r="C221" t="n">
-        <v>1.515771150588989</v>
+        <v>1.416432619094849</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="n">
-        <v>59</v>
+        <v>73</v>
       </c>
       <c r="B222" t="inlineStr">
         <is>
@@ -3315,12 +3315,12 @@
         </is>
       </c>
       <c r="C222" t="n">
-        <v>1.542001247406006</v>
+        <v>1.404842615127563</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="n">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="B223" t="inlineStr">
         <is>
@@ -3328,12 +3328,12 @@
         </is>
       </c>
       <c r="C223" t="n">
-        <v>1.513809084892273</v>
+        <v>1.427298307418823</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="n">
-        <v>61</v>
+        <v>75</v>
       </c>
       <c r="B224" t="inlineStr">
         <is>
@@ -3341,12 +3341,12 @@
         </is>
       </c>
       <c r="C224" t="n">
-        <v>1.6966632604599</v>
+        <v>1.433727025985718</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="n">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="B225" t="inlineStr">
         <is>
@@ -3354,12 +3354,12 @@
         </is>
       </c>
       <c r="C225" t="n">
-        <v>1.60943078994751</v>
+        <v>1.43722665309906</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="n">
-        <v>63</v>
+        <v>77</v>
       </c>
       <c r="B226" t="inlineStr">
         <is>
@@ -3367,12 +3367,12 @@
         </is>
       </c>
       <c r="C226" t="n">
-        <v>1.527853488922119</v>
+        <v>1.410547256469727</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="n">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="B227" t="inlineStr">
         <is>
@@ -3380,12 +3380,12 @@
         </is>
       </c>
       <c r="C227" t="n">
-        <v>1.478474378585815</v>
+        <v>1.344621419906616</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="n">
-        <v>65</v>
+        <v>79</v>
       </c>
       <c r="B228" t="inlineStr">
         <is>
@@ -3393,12 +3393,12 @@
         </is>
       </c>
       <c r="C228" t="n">
-        <v>1.549293756484985</v>
+        <v>1.403871536254883</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="n">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="B229" t="inlineStr">
         <is>
@@ -3406,12 +3406,12 @@
         </is>
       </c>
       <c r="C229" t="n">
-        <v>1.619354963302612</v>
+        <v>1.403160333633423</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="n">
-        <v>67</v>
+        <v>81</v>
       </c>
       <c r="B230" t="inlineStr">
         <is>
@@ -3419,12 +3419,12 @@
         </is>
       </c>
       <c r="C230" t="n">
-        <v>1.526079416275024</v>
+        <v>1.400931477546692</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="n">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="B231" t="inlineStr">
         <is>
@@ -3432,12 +3432,12 @@
         </is>
       </c>
       <c r="C231" t="n">
-        <v>1.594233274459839</v>
+        <v>1.524519920349121</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="n">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="B232" t="inlineStr">
         <is>
@@ -3445,12 +3445,12 @@
         </is>
       </c>
       <c r="C232" t="n">
-        <v>1.476624965667725</v>
+        <v>1.431838035583496</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="n">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="B233" t="inlineStr">
         <is>
@@ -3458,12 +3458,12 @@
         </is>
       </c>
       <c r="C233" t="n">
-        <v>1.573757171630859</v>
+        <v>1.448146104812622</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="n">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="B234" t="inlineStr">
         <is>
@@ -3471,12 +3471,12 @@
         </is>
       </c>
       <c r="C234" t="n">
-        <v>1.498879909515381</v>
+        <v>1.431792497634888</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="n">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="B235" t="inlineStr">
         <is>
@@ -3484,12 +3484,12 @@
         </is>
       </c>
       <c r="C235" t="n">
-        <v>1.653540968894958</v>
+        <v>1.525513887405396</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="n">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="B236" t="inlineStr">
         <is>
@@ -3497,12 +3497,12 @@
         </is>
       </c>
       <c r="C236" t="n">
-        <v>1.573062777519226</v>
+        <v>1.48291802406311</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="n">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="B237" t="inlineStr">
         <is>
@@ -3510,12 +3510,12 @@
         </is>
       </c>
       <c r="C237" t="n">
-        <v>1.563776969909668</v>
+        <v>1.451005935668945</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="n">
-        <v>75</v>
+        <v>89</v>
       </c>
       <c r="B238" t="inlineStr">
         <is>
@@ -3523,12 +3523,12 @@
         </is>
       </c>
       <c r="C238" t="n">
-        <v>1.510509729385376</v>
+        <v>1.532082676887512</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="n">
-        <v>76</v>
+        <v>90</v>
       </c>
       <c r="B239" t="inlineStr">
         <is>
@@ -3536,12 +3536,12 @@
         </is>
       </c>
       <c r="C239" t="n">
-        <v>1.700397968292236</v>
+        <v>1.482724189758301</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="n">
-        <v>77</v>
+        <v>91</v>
       </c>
       <c r="B240" t="inlineStr">
         <is>
@@ -3549,12 +3549,12 @@
         </is>
       </c>
       <c r="C240" t="n">
-        <v>1.580052137374878</v>
+        <v>1.434587001800537</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="n">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="B241" t="inlineStr">
         <is>
@@ -3562,12 +3562,12 @@
         </is>
       </c>
       <c r="C241" t="n">
-        <v>1.434452056884766</v>
+        <v>1.386884093284607</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="n">
-        <v>79</v>
+        <v>93</v>
       </c>
       <c r="B242" t="inlineStr">
         <is>
@@ -3575,12 +3575,12 @@
         </is>
       </c>
       <c r="C242" t="n">
-        <v>1.455438137054443</v>
+        <v>1.438125729560852</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="n">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="B243" t="inlineStr">
         <is>
@@ -3588,12 +3588,12 @@
         </is>
       </c>
       <c r="C243" t="n">
-        <v>1.599017381668091</v>
+        <v>1.464312553405762</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="n">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="B244" t="inlineStr">
         <is>
@@ -3601,12 +3601,12 @@
         </is>
       </c>
       <c r="C244" t="n">
-        <v>1.52264940738678</v>
+        <v>1.437524795532227</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="n">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="B245" t="inlineStr">
         <is>
@@ -3614,12 +3614,12 @@
         </is>
       </c>
       <c r="C245" t="n">
-        <v>1.515021562576294</v>
+        <v>1.498050928115845</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="n">
-        <v>83</v>
+        <v>97</v>
       </c>
       <c r="B246" t="inlineStr">
         <is>
@@ -3627,12 +3627,12 @@
         </is>
       </c>
       <c r="C246" t="n">
-        <v>1.542975187301636</v>
+        <v>1.481415748596191</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="n">
-        <v>84</v>
+        <v>98</v>
       </c>
       <c r="B247" t="inlineStr">
         <is>
@@ -3640,12 +3640,12 @@
         </is>
       </c>
       <c r="C247" t="n">
-        <v>1.483757257461548</v>
+        <v>1.417482972145081</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="n">
-        <v>85</v>
+        <v>99</v>
       </c>
       <c r="B248" t="inlineStr">
         <is>
@@ -3653,12 +3653,12 @@
         </is>
       </c>
       <c r="C248" t="n">
-        <v>1.511547088623047</v>
+        <v>1.405329823493958</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="n">
-        <v>86</v>
+        <v>100</v>
       </c>
       <c r="B249" t="inlineStr">
         <is>
@@ -3666,12 +3666,12 @@
         </is>
       </c>
       <c r="C249" t="n">
-        <v>1.559482216835022</v>
+        <v>1.489744901657104</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="n">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="B250" t="inlineStr">
         <is>
@@ -3679,12 +3679,12 @@
         </is>
       </c>
       <c r="C250" t="n">
-        <v>1.570040225982666</v>
+        <v>1.460583209991455</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="n">
-        <v>88</v>
+        <v>102</v>
       </c>
       <c r="B251" t="inlineStr">
         <is>
@@ -3692,12 +3692,12 @@
         </is>
       </c>
       <c r="C251" t="n">
-        <v>1.576745867729187</v>
+        <v>1.426521182060242</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="n">
-        <v>89</v>
+        <v>103</v>
       </c>
       <c r="B252" t="inlineStr">
         <is>
@@ -3705,12 +3705,12 @@
         </is>
       </c>
       <c r="C252" t="n">
-        <v>1.43869423866272</v>
+        <v>1.412698268890381</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="n">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="B253" t="inlineStr">
         <is>
@@ -3718,12 +3718,12 @@
         </is>
       </c>
       <c r="C253" t="n">
-        <v>1.573304414749146</v>
+        <v>1.404993295669556</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="n">
-        <v>91</v>
+        <v>105</v>
       </c>
       <c r="B254" t="inlineStr">
         <is>
@@ -3731,12 +3731,12 @@
         </is>
       </c>
       <c r="C254" t="n">
-        <v>1.520442247390747</v>
+        <v>1.396716356277466</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="n">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="B255" t="inlineStr">
         <is>
@@ -3744,12 +3744,12 @@
         </is>
       </c>
       <c r="C255" t="n">
-        <v>1.542507290840149</v>
+        <v>1.383261919021606</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="n">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="B256" t="inlineStr">
         <is>
@@ -3757,12 +3757,12 @@
         </is>
       </c>
       <c r="C256" t="n">
-        <v>1.563115119934082</v>
+        <v>1.327399134635925</v>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="n">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="B257" t="inlineStr">
         <is>
@@ -3770,12 +3770,12 @@
         </is>
       </c>
       <c r="C257" t="n">
-        <v>1.511996030807495</v>
+        <v>1.417009592056274</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="n">
-        <v>95</v>
+        <v>109</v>
       </c>
       <c r="B258" t="inlineStr">
         <is>
@@ -3783,12 +3783,12 @@
         </is>
       </c>
       <c r="C258" t="n">
-        <v>1.639196872711182</v>
+        <v>1.306456565856934</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="n">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="B259" t="inlineStr">
         <is>
@@ -3796,12 +3796,12 @@
         </is>
       </c>
       <c r="C259" t="n">
-        <v>1.516765117645264</v>
+        <v>1.422800302505493</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="n">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="B260" t="inlineStr">
         <is>
@@ -3809,12 +3809,12 @@
         </is>
       </c>
       <c r="C260" t="n">
-        <v>1.571464061737061</v>
+        <v>1.37656569480896</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="n">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="B261" t="inlineStr">
         <is>
@@ -3822,12 +3822,12 @@
         </is>
       </c>
       <c r="C261" t="n">
-        <v>1.526957035064697</v>
+        <v>1.420188665390015</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="n">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="B262" t="inlineStr">
         <is>
@@ -3835,12 +3835,12 @@
         </is>
       </c>
       <c r="C262" t="n">
-        <v>1.534288048744202</v>
+        <v>1.417806267738342</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="n">
-        <v>100</v>
+        <v>114</v>
       </c>
       <c r="B263" t="inlineStr">
         <is>
@@ -3848,12 +3848,12 @@
         </is>
       </c>
       <c r="C263" t="n">
-        <v>1.548850059509277</v>
+        <v>1.444743394851685</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="n">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="B264" t="inlineStr">
         <is>
@@ -3861,12 +3861,12 @@
         </is>
       </c>
       <c r="C264" t="n">
-        <v>1.530040740966797</v>
+        <v>1.467926383018494</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="n">
-        <v>102</v>
+        <v>116</v>
       </c>
       <c r="B265" t="inlineStr">
         <is>
@@ -3874,12 +3874,12 @@
         </is>
       </c>
       <c r="C265" t="n">
-        <v>1.599879741668701</v>
+        <v>1.449906349182129</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="n">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="B266" t="inlineStr">
         <is>
@@ -3887,12 +3887,12 @@
         </is>
       </c>
       <c r="C266" t="n">
-        <v>1.587548017501831</v>
+        <v>1.405207753181458</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="n">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="B267" t="inlineStr">
         <is>
@@ -3900,12 +3900,12 @@
         </is>
       </c>
       <c r="C267" t="n">
-        <v>1.482994794845581</v>
+        <v>1.390084505081177</v>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="n">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="B268" t="inlineStr">
         <is>
@@ -3913,12 +3913,12 @@
         </is>
       </c>
       <c r="C268" t="n">
-        <v>1.533520698547363</v>
+        <v>1.425193548202515</v>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="n">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="B269" t="inlineStr">
         <is>
@@ -3926,12 +3926,12 @@
         </is>
       </c>
       <c r="C269" t="n">
-        <v>1.516415238380432</v>
+        <v>1.379063606262207</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="n">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="B270" t="inlineStr">
         <is>
@@ -3939,12 +3939,12 @@
         </is>
       </c>
       <c r="C270" t="n">
-        <v>1.523113012313843</v>
+        <v>1.404829144477844</v>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="n">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="B271" t="inlineStr">
         <is>
@@ -3952,12 +3952,12 @@
         </is>
       </c>
       <c r="C271" t="n">
-        <v>1.493738174438477</v>
+        <v>1.454021453857422</v>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="n">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="B272" t="inlineStr">
         <is>
@@ -3965,12 +3965,12 @@
         </is>
       </c>
       <c r="C272" t="n">
-        <v>1.627955317497253</v>
+        <v>1.424896955490112</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="n">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="B273" t="inlineStr">
         <is>
@@ -3978,12 +3978,12 @@
         </is>
       </c>
       <c r="C273" t="n">
-        <v>1.529908657073975</v>
+        <v>1.3933265209198</v>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="n">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="B274" t="inlineStr">
         <is>
@@ -3991,12 +3991,12 @@
         </is>
       </c>
       <c r="C274" t="n">
-        <v>1.5345778465271</v>
+        <v>1.487506151199341</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="n">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="B275" t="inlineStr">
         <is>
@@ -4004,12 +4004,12 @@
         </is>
       </c>
       <c r="C275" t="n">
-        <v>1.495252370834351</v>
+        <v>1.432717084884644</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="n">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="B276" t="inlineStr">
         <is>
@@ -4017,12 +4017,12 @@
         </is>
       </c>
       <c r="C276" t="n">
-        <v>1.521043062210083</v>
+        <v>1.440849542617798</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="n">
-        <v>114</v>
+        <v>128</v>
       </c>
       <c r="B277" t="inlineStr">
         <is>
@@ -4030,12 +4030,12 @@
         </is>
       </c>
       <c r="C277" t="n">
-        <v>1.540778756141663</v>
+        <v>1.458962082862854</v>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="n">
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="B278" t="inlineStr">
         <is>
@@ -4043,12 +4043,12 @@
         </is>
       </c>
       <c r="C278" t="n">
-        <v>1.53505802154541</v>
+        <v>1.403688788414001</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="n">
-        <v>116</v>
+        <v>130</v>
       </c>
       <c r="B279" t="inlineStr">
         <is>
@@ -4056,12 +4056,12 @@
         </is>
       </c>
       <c r="C279" t="n">
-        <v>1.499051332473755</v>
+        <v>1.522887945175171</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="n">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="B280" t="inlineStr">
         <is>
@@ -4069,12 +4069,12 @@
         </is>
       </c>
       <c r="C280" t="n">
-        <v>1.480635046958923</v>
+        <v>1.388452053070068</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="n">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="B281" t="inlineStr">
         <is>
@@ -4082,12 +4082,12 @@
         </is>
       </c>
       <c r="C281" t="n">
-        <v>1.564874172210693</v>
+        <v>1.388243079185486</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="n">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="B282" t="inlineStr">
         <is>
@@ -4095,12 +4095,12 @@
         </is>
       </c>
       <c r="C282" t="n">
-        <v>1.586597204208374</v>
+        <v>1.428824901580811</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="n">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="B283" t="inlineStr">
         <is>
@@ -4108,12 +4108,12 @@
         </is>
       </c>
       <c r="C283" t="n">
-        <v>1.538365721702576</v>
+        <v>1.490392208099365</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="n">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="B284" t="inlineStr">
         <is>
@@ -4121,12 +4121,12 @@
         </is>
       </c>
       <c r="C284" t="n">
-        <v>1.568626403808594</v>
+        <v>1.486376523971558</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="n">
-        <v>122</v>
+        <v>136</v>
       </c>
       <c r="B285" t="inlineStr">
         <is>
@@ -4134,12 +4134,12 @@
         </is>
       </c>
       <c r="C285" t="n">
-        <v>1.51521897315979</v>
+        <v>1.351970911026001</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="n">
-        <v>123</v>
+        <v>137</v>
       </c>
       <c r="B286" t="inlineStr">
         <is>
@@ -4147,12 +4147,12 @@
         </is>
       </c>
       <c r="C286" t="n">
-        <v>1.592950224876404</v>
+        <v>1.412788867950439</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="n">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="B287" t="inlineStr">
         <is>
@@ -4160,12 +4160,12 @@
         </is>
       </c>
       <c r="C287" t="n">
-        <v>1.516898155212402</v>
+        <v>1.439483642578125</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="n">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="B288" t="inlineStr">
         <is>
@@ -4173,12 +4173,12 @@
         </is>
       </c>
       <c r="C288" t="n">
-        <v>1.47965931892395</v>
+        <v>1.395126342773438</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="n">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="B289" t="inlineStr">
         <is>
@@ -4186,12 +4186,12 @@
         </is>
       </c>
       <c r="C289" t="n">
-        <v>1.521347761154175</v>
+        <v>1.41877555847168</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="n">
-        <v>127</v>
+        <v>141</v>
       </c>
       <c r="B290" t="inlineStr">
         <is>
@@ -4199,12 +4199,12 @@
         </is>
       </c>
       <c r="C290" t="n">
-        <v>1.59260106086731</v>
+        <v>1.404404520988464</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="n">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="B291" t="inlineStr">
         <is>
@@ -4212,12 +4212,12 @@
         </is>
       </c>
       <c r="C291" t="n">
-        <v>1.473366737365723</v>
+        <v>1.397712826728821</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="n">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="B292" t="inlineStr">
         <is>
@@ -4225,12 +4225,12 @@
         </is>
       </c>
       <c r="C292" t="n">
-        <v>1.463700771331787</v>
+        <v>1.315837621688843</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="n">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="B293" t="inlineStr">
         <is>
@@ -4238,12 +4238,12 @@
         </is>
       </c>
       <c r="C293" t="n">
-        <v>1.480927705764771</v>
+        <v>1.232426047325134</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="n">
-        <v>131</v>
+        <v>145</v>
       </c>
       <c r="B294" t="inlineStr">
         <is>
@@ -4251,12 +4251,12 @@
         </is>
       </c>
       <c r="C294" t="n">
-        <v>1.601182222366333</v>
+        <v>1.078904747962952</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="B295" t="inlineStr">
         <is>
@@ -4264,12 +4264,12 @@
         </is>
       </c>
       <c r="C295" t="n">
-        <v>1.532884359359741</v>
+        <v>1.032259941101074</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="n">
-        <v>133</v>
+        <v>147</v>
       </c>
       <c r="B296" t="inlineStr">
         <is>
@@ -4277,384 +4277,7 @@
         </is>
       </c>
       <c r="C296" t="n">
-        <v>1.68381679058075</v>
-      </c>
-    </row>
-    <row r="297">
-      <c r="A297" t="n">
-        <v>134</v>
-      </c>
-      <c r="B297" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C297" t="n">
-        <v>1.728768229484558</v>
-      </c>
-    </row>
-    <row r="298">
-      <c r="A298" t="n">
-        <v>135</v>
-      </c>
-      <c r="B298" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C298" t="n">
-        <v>1.679852724075317</v>
-      </c>
-    </row>
-    <row r="299">
-      <c r="A299" t="n">
-        <v>136</v>
-      </c>
-      <c r="B299" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C299" t="n">
-        <v>1.63956344127655</v>
-      </c>
-    </row>
-    <row r="300">
-      <c r="A300" t="n">
-        <v>137</v>
-      </c>
-      <c r="B300" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C300" t="n">
-        <v>1.584820628166199</v>
-      </c>
-    </row>
-    <row r="301">
-      <c r="A301" t="n">
-        <v>138</v>
-      </c>
-      <c r="B301" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C301" t="n">
-        <v>1.53381872177124</v>
-      </c>
-    </row>
-    <row r="302">
-      <c r="A302" t="n">
-        <v>139</v>
-      </c>
-      <c r="B302" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C302" t="n">
-        <v>1.623190402984619</v>
-      </c>
-    </row>
-    <row r="303">
-      <c r="A303" t="n">
-        <v>140</v>
-      </c>
-      <c r="B303" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C303" t="n">
-        <v>1.526060819625854</v>
-      </c>
-    </row>
-    <row r="304">
-      <c r="A304" t="n">
-        <v>141</v>
-      </c>
-      <c r="B304" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C304" t="n">
-        <v>1.617721438407898</v>
-      </c>
-    </row>
-    <row r="305">
-      <c r="A305" t="n">
-        <v>142</v>
-      </c>
-      <c r="B305" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C305" t="n">
-        <v>1.564908146858215</v>
-      </c>
-    </row>
-    <row r="306">
-      <c r="A306" t="n">
-        <v>143</v>
-      </c>
-      <c r="B306" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C306" t="n">
-        <v>1.662998199462891</v>
-      </c>
-    </row>
-    <row r="307">
-      <c r="A307" t="n">
-        <v>144</v>
-      </c>
-      <c r="B307" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C307" t="n">
-        <v>1.61133337020874</v>
-      </c>
-    </row>
-    <row r="308">
-      <c r="A308" t="n">
-        <v>145</v>
-      </c>
-      <c r="B308" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C308" t="n">
-        <v>1.510688424110413</v>
-      </c>
-    </row>
-    <row r="309">
-      <c r="A309" t="n">
-        <v>146</v>
-      </c>
-      <c r="B309" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C309" t="n">
-        <v>1.411666393280029</v>
-      </c>
-    </row>
-    <row r="310">
-      <c r="A310" t="n">
-        <v>147</v>
-      </c>
-      <c r="B310" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C310" t="n">
-        <v>1.58565890789032</v>
-      </c>
-    </row>
-    <row r="311">
-      <c r="A311" t="n">
-        <v>148</v>
-      </c>
-      <c r="B311" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C311" t="n">
-        <v>1.721941113471985</v>
-      </c>
-    </row>
-    <row r="312">
-      <c r="A312" t="n">
-        <v>149</v>
-      </c>
-      <c r="B312" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C312" t="n">
-        <v>1.61872136592865</v>
-      </c>
-    </row>
-    <row r="313">
-      <c r="A313" t="n">
-        <v>150</v>
-      </c>
-      <c r="B313" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C313" t="n">
-        <v>1.513037443161011</v>
-      </c>
-    </row>
-    <row r="314">
-      <c r="A314" t="n">
-        <v>151</v>
-      </c>
-      <c r="B314" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C314" t="n">
-        <v>1.456647515296936</v>
-      </c>
-    </row>
-    <row r="315">
-      <c r="A315" t="n">
-        <v>152</v>
-      </c>
-      <c r="B315" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C315" t="n">
-        <v>1.643019199371338</v>
-      </c>
-    </row>
-    <row r="316">
-      <c r="A316" t="n">
-        <v>153</v>
-      </c>
-      <c r="B316" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C316" t="n">
-        <v>1.563819885253906</v>
-      </c>
-    </row>
-    <row r="317">
-      <c r="A317" t="n">
-        <v>154</v>
-      </c>
-      <c r="B317" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C317" t="n">
-        <v>1.56766140460968</v>
-      </c>
-    </row>
-    <row r="318">
-      <c r="A318" t="n">
-        <v>155</v>
-      </c>
-      <c r="B318" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C318" t="n">
-        <v>1.571278691291809</v>
-      </c>
-    </row>
-    <row r="319">
-      <c r="A319" t="n">
-        <v>156</v>
-      </c>
-      <c r="B319" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C319" t="n">
-        <v>1.494381904602051</v>
-      </c>
-    </row>
-    <row r="320">
-      <c r="A320" t="n">
-        <v>157</v>
-      </c>
-      <c r="B320" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C320" t="n">
-        <v>1.622586727142334</v>
-      </c>
-    </row>
-    <row r="321">
-      <c r="A321" t="n">
-        <v>158</v>
-      </c>
-      <c r="B321" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C321" t="n">
-        <v>1.367429256439209</v>
-      </c>
-    </row>
-    <row r="322">
-      <c r="A322" t="n">
-        <v>159</v>
-      </c>
-      <c r="B322" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C322" t="n">
-        <v>1.061538219451904</v>
-      </c>
-    </row>
-    <row r="323">
-      <c r="A323" t="n">
-        <v>160</v>
-      </c>
-      <c r="B323" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C323" t="n">
-        <v>1.044332265853882</v>
-      </c>
-    </row>
-    <row r="324">
-      <c r="A324" t="n">
-        <v>161</v>
-      </c>
-      <c r="B324" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C324" t="n">
-        <v>0.9656334519386292</v>
-      </c>
-    </row>
-    <row r="325">
-      <c r="A325" t="n">
-        <v>162</v>
-      </c>
-      <c r="B325" t="inlineStr">
-        <is>
-          <t>right</t>
-        </is>
-      </c>
-      <c r="C325" t="n">
-        <v>1.04241681098938</v>
+        <v>0.9643154144287109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>